<commit_message>
(Re)adding input files for VOCs and PFAS.
</commit_message>
<xml_diff>
--- a/Inputs/MeOH_template_parameters_Exposure.xlsx
+++ b/Inputs/MeOH_template_parameters_Exposure.xlsx
@@ -6759,7 +6759,6 @@
     <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </j747ac98061d40f0aa7bd47e1db5675d>
-    <Records_x0020_Status xmlns="93237db7-bebb-43bb-9414-bc3313990c09">Pending</Records_x0020_Status>
     <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
     <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -6786,8 +6785,13 @@
         <AccountType/>
       </UserInfo>
     </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <Records_x0020_Date xmlns="93237db7-bebb-43bb-9414-bc3313990c09" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
 </file>
@@ -6807,49 +6811,53 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010031E6F7E14DB9F64AA435011CFD87FE7C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c974ac748e8c5d1a2dbcb03dc7039540">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns4="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns5="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns6="8686fd38-6384-41df-bf60-a073971185a6" xmlns:ns7="93237db7-bebb-43bb-9414-bc3313990c09" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e31f61be74db07117ec521e527c7dfb9" ns1:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="" ns7:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint.v3"/>
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <xsd:import namespace="8686fd38-6384-41df-bf60-a073971185a6"/>
-    <xsd:import namespace="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <xsd:import namespace="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <xsd:import namespace="41d9f072-86bf-4c63-b117-debf50ff4701"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
-                <xsd:element ref="ns3:Document_x0020_Creation_x0020_Date" minOccurs="0"/>
-                <xsd:element ref="ns3:Creator" minOccurs="0"/>
-                <xsd:element ref="ns3:EPA_x0020_Office" minOccurs="0"/>
-                <xsd:element ref="ns3:Record" minOccurs="0"/>
-                <xsd:element ref="ns4:CategoryDescription" minOccurs="0"/>
-                <xsd:element ref="ns3:Identifier" minOccurs="0"/>
-                <xsd:element ref="ns3:EPA_x0020_Contributor" minOccurs="0"/>
-                <xsd:element ref="ns3:External_x0020_Contributor" minOccurs="0"/>
-                <xsd:element ref="ns5:_Coverage" minOccurs="0"/>
-                <xsd:element ref="ns3:EPA_x0020_Related_x0020_Documents" minOccurs="0"/>
-                <xsd:element ref="ns5:_Source" minOccurs="0"/>
-                <xsd:element ref="ns3:Rights" minOccurs="0"/>
+                <xsd:element ref="ns2:Document_x0020_Creation_x0020_Date" minOccurs="0"/>
+                <xsd:element ref="ns2:Creator" minOccurs="0"/>
+                <xsd:element ref="ns2:EPA_x0020_Office" minOccurs="0"/>
+                <xsd:element ref="ns2:Record" minOccurs="0"/>
+                <xsd:element ref="ns3:CategoryDescription" minOccurs="0"/>
+                <xsd:element ref="ns2:Identifier" minOccurs="0"/>
+                <xsd:element ref="ns2:EPA_x0020_Contributor" minOccurs="0"/>
+                <xsd:element ref="ns2:External_x0020_Contributor" minOccurs="0"/>
+                <xsd:element ref="ns4:_Coverage" minOccurs="0"/>
+                <xsd:element ref="ns2:EPA_x0020_Related_x0020_Documents" minOccurs="0"/>
+                <xsd:element ref="ns4:_Source" minOccurs="0"/>
+                <xsd:element ref="ns2:Rights" minOccurs="0"/>
                 <xsd:element ref="ns1:Language" minOccurs="0"/>
-                <xsd:element ref="ns3:j747ac98061d40f0aa7bd47e1db5675d" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxKeywordTaxHTField" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAllLabel" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns6:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns7:Records_x0020_Status" minOccurs="0"/>
-                <xsd:element ref="ns7:Records_x0020_Date" minOccurs="0"/>
-                <xsd:element ref="ns7:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns7:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns7:SharingHintHash" minOccurs="0"/>
+                <xsd:element ref="ns2:j747ac98061d40f0aa7bd47e1db5675d" minOccurs="0"/>
+                <xsd:element ref="ns2:TaxKeywordTaxHTField" minOccurs="0"/>
+                <xsd:element ref="ns2:TaxCatchAllLabel" minOccurs="0"/>
+                <xsd:element ref="ns2:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:e3f09c3df709400db2417a7161762d62" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns6:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns6:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns5:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns5:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -6942,7 +6950,7 @@
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="Record" ma:index="5" nillable="true" ma:displayName="Record" ma:default="Shared" ma:description="For documents that provide evidence of EPA decisions and actions, select &quot;Shared&quot; (open access) or &quot;Private&quot; (restricted access)." ma:format="Dropdown" ma:internalName="Record">
+    <xsd:element name="Record" ma:index="5" nillable="true" ma:displayName="Record" ma:default="Shared" ma:description="For documents that provide evidence of EPA decisions and actions, select &quot;Shared&quot; (open access) or &quot;Private&quot; (restricted access)." ma:format="Dropdown" ma:internalName="Record" ma:readOnly="false">
       <xsd:simpleType>
         <xsd:restriction base="dms:Choice">
           <xsd:enumeration value="None"/>
@@ -7012,7 +7020,7 @@
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="TaxCatchAllLabel" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column1" ma:hidden="true" ma:list="{a37802d4-57e0-410e-a276-34e3d7c16864}" ma:internalName="TaxCatchAllLabel" ma:readOnly="true" ma:showField="CatchAllDataLabel" ma:web="93237db7-bebb-43bb-9414-bc3313990c09">
+    <xsd:element name="TaxCatchAllLabel" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column1" ma:description="" ma:hidden="true" ma:list="{3f8140d4-46ad-4523-b80f-0b31c25fa229}" ma:internalName="TaxCatchAllLabel" ma:readOnly="true" ma:showField="CatchAllDataLabel" ma:web="41d9f072-86bf-4c63-b117-debf50ff4701">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -7023,7 +7031,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="24" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{a37802d4-57e0-410e-a276-34e3d7c16864}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="93237db7-bebb-43bb-9414-bc3313990c09">
+    <xsd:element name="TaxCatchAll" ma:index="24" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:description="" ma:hidden="true" ma:list="{3f8140d4-46ad-4523-b80f-0b31c25fa229}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="41d9f072-86bf-4c63-b117-debf50ff4701">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -7032,6 +7040,13 @@
             </xsd:sequence>
           </xsd:extension>
         </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="e3f09c3df709400db2417a7161762d62" ma:index="28" nillable="true" ma:taxonomy="true" ma:internalName="e3f09c3df709400db2417a7161762d62" ma:taxonomyFieldName="EPA_x0020_Subject" ma:displayName="EPA Subject" ma:readOnly="false" ma:default="" ma:fieldId="{e3f09c3d-f709-400d-b241-7a7161762d62}" ma:taxonomyMulti="true" ma:sspId="29f62856-1543-49d4-a736-4569d363f533" ma:termSetId="7a3d4ae0-7e62-45a2-a406-c6a8a6a8eee3" ma:anchorId="00000000-0000-0000-0000-000000000000" ma:open="false" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
@@ -7064,61 +7079,85 @@
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8686fd38-6384-41df-bf60-a073971185a6" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2ba80736-48fa-4d73-aaff-bacaeeed013a" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="28" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceMetadata" ma:index="29" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="29" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceFastMetadata" ma:index="30" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="30" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoTags" ma:index="31" nillable="true" ma:displayName="MediaServiceAutoTags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="31" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="32" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="33" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="34" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="32" nillable="true" ma:displayName="MediaServiceOCR" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="93237db7-bebb-43bb-9414-bc3313990c09" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="Records_x0020_Status" ma:index="35" nillable="true" ma:displayName="Records Status" ma:default="Pending" ma:internalName="Records_x0020_Status">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="35" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="Records_x0020_Date" ma:index="36" nillable="true" ma:displayName="Records Date" ma:hidden="true" ma:internalName="Records_x0020_Date">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="36" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="37" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="37" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="38" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="39" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="41" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="29f62856-1543-49d4-a736-4569d363f533" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="42" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="43" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="44" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="41d9f072-86bf-4c63-b117-debf50ff4701" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="33" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -7137,16 +7176,11 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="38" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="34" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="SharingHintHash" ma:index="39" nillable="true" ma:displayName="Sharing Hint Hash" ma:hidden="true" ma:internalName="SharingHintHash" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -7280,24 +7314,5 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D47D7CD8-1E46-46BB-A82A-284BAE4E7E0E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="8686fd38-6384-41df-bf60-a073971185a6"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE4635F4-476B-45CA-B487-8C40A4AECF43}"/>
 </file>
</xml_diff>